<commit_message>
modify mechanical design materials
</commit_message>
<xml_diff>
--- a/mechanical/screw_list.xlsx
+++ b/mechanical/screw_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lipoy\Dropbox\develop\Sense-chan\Sense-chan\mechanical\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C032E6D5-3615-4C40-8EDB-09F624530345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAD1E1F-CD09-4FD3-AF1D-235087E65B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>使用箇所</t>
     <rPh sb="0" eb="4">
@@ -635,6 +635,9 @@
       <c r="D7" s="1">
         <v>8</v>
       </c>
+      <c r="E7" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">

</xml_diff>